<commit_message>
compute kpis via sql instead of excel formulas
</commit_message>
<xml_diff>
--- a/examples/export-example.xlsx
+++ b/examples/export-example.xlsx
@@ -124,7 +124,7 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>2026-07-04 15:33:57</t>
+          <t>2026-07-04 19:28:04</t>
         </is>
       </c>
     </row>
@@ -217,7 +217,7 @@
         </is>
       </c>
       <c r="B2" s="0">
-        <f>COUNTA('Players'!A2:A100000)</f>
+        <v>150</v>
       </c>
       <c r="C2" s="0" t="inlineStr">
         <is>
@@ -232,7 +232,7 @@
         </is>
       </c>
       <c r="B3" s="0">
-        <f>COUNTIF('Players'!K2:K100000,"completed")</f>
+        <v>99</v>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
@@ -247,7 +247,7 @@
         </is>
       </c>
       <c r="B4" s="0">
-        <f>IF(B2=0,0,B3/B2)</f>
+        <v>0.66</v>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
@@ -262,11 +262,11 @@
         </is>
       </c>
       <c r="B5" s="0">
-        <f>SUM('Players'!G2:G100000)</f>
+        <v>1513455</v>
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>Somma score</t>
+          <t>Somma payload.score</t>
         </is>
       </c>
     </row>
@@ -277,26 +277,26 @@
         </is>
       </c>
       <c r="B6" s="0">
-        <f>AVERAGE('Players'!G2:G100000)</f>
+        <v>10089.7</v>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>Media score</t>
+          <t>Score totale / player</t>
         </is>
       </c>
     </row>
     <row r="7" spans="1:3" customHeight="0">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>Eventi totali aggregati</t>
+          <t>Eventi totali</t>
         </is>
       </c>
       <c r="B7" s="0">
-        <f>SUM('Events_Summary'!D2:D100000)</f>
+        <v>3000</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>Somma eventi aggregati</t>
+          <t>Conteggio eventi</t>
         </is>
       </c>
     </row>
@@ -307,7 +307,7 @@
         </is>
       </c>
       <c r="B8" s="0">
-        <f>COUNTA('Transactions'!A2:A100000)</f>
+        <v>147</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
@@ -322,7 +322,7 @@
         </is>
       </c>
       <c r="B9" s="0">
-        <f>SUM('Transactions'!E2:E100000)</f>
+        <v>14570.64</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
@@ -337,11 +337,11 @@
         </is>
       </c>
       <c r="B10" s="0">
-        <f>SUM('Answers'!D2:D100000)</f>
+        <v>256</v>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>Somma risposte</t>
+          <t>Conteggio risposte</t>
         </is>
       </c>
     </row>
@@ -352,11 +352,11 @@
         </is>
       </c>
       <c r="B11" s="0">
-        <f>SUMIF('Data_Quality'!B2:B100000,"error",'Data_Quality'!C2:C100000)</f>
+        <v>607</v>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t>Somma anomalie error</t>
+          <t>Anomalie di severita error</t>
         </is>
       </c>
     </row>
@@ -13843,47 +13843,47 @@
     <row r="3" spans="1:5" customHeight="0">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t>q2</t>
+          <t>q1</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>Question 2</t>
+          <t>Question 1</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>Answer 3</t>
+          <t>Answer 2</t>
         </is>
       </c>
       <c r="D3" s="0">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E3" s="0">
-        <v>0.1724</v>
+        <v>0.314</v>
       </c>
     </row>
     <row r="4" spans="1:5" customHeight="0">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t>q3</t>
+          <t>q1</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>Question 3</t>
+          <t>Question 1</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>Answer 3</t>
+          <t>Answer 4</t>
         </is>
       </c>
       <c r="D4" s="0">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="E4" s="0">
-        <v>0.3125</v>
+        <v>0.2727</v>
       </c>
     </row>
     <row r="5" spans="1:5" customHeight="0">
@@ -13899,14 +13899,14 @@
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>Answer 2</t>
+          <t>Answer 3</t>
         </is>
       </c>
       <c r="D5" s="0">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="E5" s="0">
-        <v>0.314</v>
+        <v>0.2149</v>
       </c>
     </row>
     <row r="6" spans="1:5" customHeight="0">
@@ -13922,48 +13922,48 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>Answer 1</t>
+          <t>Answer 3</t>
         </is>
       </c>
       <c r="D6" s="0">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="E6" s="0">
-        <v>0.2989</v>
+        <v>0.1724</v>
       </c>
     </row>
     <row r="7" spans="1:5" customHeight="0">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>q3</t>
+          <t>q2</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>Question 3</t>
+          <t>Question 2</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>Answer 4</t>
+          <t>Answer 1</t>
         </is>
       </c>
       <c r="D7" s="0">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="E7" s="0">
-        <v>0.2292</v>
+        <v>0.2989</v>
       </c>
     </row>
     <row r="8" spans="1:5" customHeight="0">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>q1</t>
+          <t>q2</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>Question 1</t>
+          <t>Question 2</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -13972,21 +13972,21 @@
         </is>
       </c>
       <c r="D8" s="0">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E8" s="0">
-        <v>0.2727</v>
+        <v>0.3103</v>
       </c>
     </row>
     <row r="9" spans="1:5" customHeight="0">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>q3</t>
+          <t>q2</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>Question 3</t>
+          <t>Question 2</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -13995,33 +13995,33 @@
         </is>
       </c>
       <c r="D9" s="0">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="E9" s="0">
-        <v>0.1458</v>
+        <v>0.2184</v>
       </c>
     </row>
     <row r="10" spans="1:5" customHeight="0">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>q2</t>
+          <t>q3</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>Question 2</t>
+          <t>Question 3</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>Answer 4</t>
+          <t>Answer 3</t>
         </is>
       </c>
       <c r="D10" s="0">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="E10" s="0">
-        <v>0.3103</v>
+        <v>0.3125</v>
       </c>
     </row>
     <row r="11" spans="1:5" customHeight="0">
@@ -14037,60 +14037,60 @@
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t>Answer 1</t>
+          <t>Answer 4</t>
         </is>
       </c>
       <c r="D11" s="0">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E11" s="0">
-        <v>0.3125</v>
+        <v>0.2292</v>
       </c>
     </row>
     <row r="12" spans="1:5" customHeight="0">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>q1</t>
+          <t>q3</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>Question 1</t>
+          <t>Question 3</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>Answer 3</t>
+          <t>Answer 2</t>
         </is>
       </c>
       <c r="D12" s="0">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E12" s="0">
-        <v>0.2149</v>
+        <v>0.1458</v>
       </c>
     </row>
     <row r="13" spans="1:5" customHeight="0">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>q2</t>
+          <t>q3</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>Question 2</t>
+          <t>Question 3</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t>Answer 2</t>
+          <t>Answer 1</t>
         </is>
       </c>
       <c r="D13" s="0">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E13" s="0">
-        <v>0.2184</v>
+        <v>0.3125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>